<commit_message>
Finished with hypothesis testing. Added 3 exercises.
</commit_message>
<xml_diff>
--- a/resources/Part_3_Statistics/S20_L134/4.9.Test-for-the-mean.Independent-samples-Part-2-exercise-2.xlsx
+++ b/resources/Part_3_Statistics/S20_L134/4.9.Test-for-the-mean.Independent-samples-Part-2-exercise-2.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21126"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA81E69-6FA9-45AE-8FEC-C75CF3B0D44E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8988" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8985"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="179021"/>
+  <calcPr calcId="162913"/>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Mean</t>
   </si>
@@ -59,15 +58,45 @@
   </si>
   <si>
     <t>You have data on the amount of times people click on a pop-up add on 24 Mondays and 21 Saturdays on an e-learning platform for several years. The samples are drawn independently.</t>
+  </si>
+  <si>
+    <t>Pooled</t>
+  </si>
+  <si>
+    <t>Variance</t>
+  </si>
+  <si>
+    <t>Std Error</t>
+  </si>
+  <si>
+    <t>T-factor</t>
+  </si>
+  <si>
+    <t>Hypothesis:</t>
+  </si>
+  <si>
+    <t>Clicks on Monday are equal or lower than on Saturdays</t>
+  </si>
+  <si>
+    <t>Cm &lt;= Cs</t>
+  </si>
+  <si>
+    <t>Cm - Cs &lt;= 0</t>
+  </si>
+  <si>
+    <t>p-value</t>
+  </si>
+  <si>
+    <t>No, there is no evidence that the clicsk are more on Monday than on Saturday.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -159,7 +188,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -170,12 +199,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -187,7 +216,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -465,34 +494,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V23"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B3" s="2"/>
       <c r="C3" s="17" t="s">
         <v>10</v>
@@ -517,7 +546,7 @@
       <c r="U3" s="18"/>
       <c r="V3" s="18"/>
     </row>
-    <row r="4" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
@@ -542,7 +571,7 @@
       <c r="U4" s="18"/>
       <c r="V4" s="18"/>
     </row>
-    <row r="5" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
@@ -550,7 +579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B6" s="2"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.2">
@@ -559,7 +588,7 @@
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
     </row>
-    <row r="8" spans="1:22" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
@@ -576,7 +605,7 @@
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
     </row>
-    <row r="9" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" s="8"/>
       <c r="B9" s="2" t="s">
         <v>0</v>
@@ -587,9 +616,19 @@
       <c r="D9" s="12">
         <v>908.2</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="K9" s="2"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="15"/>
+      <c r="L9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>18</v>
+      </c>
       <c r="N9" s="11"/>
       <c r="O9" s="11"/>
       <c r="P9" s="11"/>
@@ -597,7 +636,7 @@
       <c r="R9" s="11"/>
       <c r="S9" s="11"/>
     </row>
-    <row r="10" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>
       <c r="B10" s="2" t="s">
         <v>1</v>
@@ -618,7 +657,7 @@
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
     </row>
-    <row r="11" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="5" t="s">
         <v>2</v>
@@ -638,7 +677,7 @@
       <c r="R11" s="11"/>
       <c r="S11" s="11"/>
     </row>
-    <row r="12" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="D12" s="13"/>
@@ -653,9 +692,11 @@
       <c r="R12" s="11"/>
       <c r="S12" s="11"/>
     </row>
-    <row r="13" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
+      <c r="B13" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
@@ -668,12 +709,20 @@
       <c r="R13" s="11"/>
       <c r="S13" s="11"/>
     </row>
-    <row r="14" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2">
+        <f>((C11-1)*(C10^2)+(D11-1)*(D10^2))/(C11+D11-2)</f>
+        <v>316978.78604651167</v>
+      </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
+      <c r="F14" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
@@ -683,26 +732,40 @@
       <c r="R14" s="11"/>
       <c r="S14" s="11"/>
     </row>
-    <row r="15" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="2"/>
+      <c r="B15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2">
+        <f>SQRT(C14/C11+C14/D11)</f>
+        <v>168.23102367156125</v>
+      </c>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
       <c r="J15" s="2"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:22" ht="12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="2">
+        <f>(C9-D9)/C15</f>
+        <v>1.0093263198083002</v>
+      </c>
       <c r="D16" s="6"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:13" ht="12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
+      <c r="B17" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="9">
+        <v>0.15923799999999999</v>
+      </c>
       <c r="D17" s="8"/>
       <c r="M17" s="2"/>
     </row>
@@ -712,7 +775,7 @@
       <c r="C18" s="9"/>
       <c r="D18" s="8"/>
     </row>
-    <row r="19" spans="1:13" ht="12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -725,7 +788,7 @@
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
     </row>
-    <row r="21" spans="1:13" ht="12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -738,7 +801,7 @@
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
     </row>
-    <row r="23" spans="1:13" ht="12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="M23" s="2"/>
     </row>
   </sheetData>

</xml_diff>